<commit_message>
Added levoglucosan uptake curve to dist example
</commit_message>
<xml_diff>
--- a/dist/example/uptake_curve.xlsx
+++ b/dist/example/uptake_curve.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mail\CLionProjects\0d_adsorption\dist\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E266B1-594E-40B7-AF55-A00889A5D2AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4118FF5-B7E0-497E-B48B-583B0B823A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17640" yWindow="2715" windowWidth="16770" windowHeight="15345" xr2:uid="{F42F43B3-C9C7-49B5-A63B-84B6B370C241}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{F42F43B3-C9C7-49B5-A63B-84B6B370C241}"/>
   </bookViews>
   <sheets>
-    <sheet name="NaCl-2" sheetId="1" r:id="rId1"/>
+    <sheet name="levoglucosan" sheetId="2" r:id="rId1"/>
+    <sheet name="NaCl-2" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
   <si>
     <t>time</t>
   </si>
@@ -64,12 +65,15 @@
   <si>
     <t>D, cm</t>
   </si>
+  <si>
+    <t>L</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,6 +104,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -122,7 +133,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -134,9 +145,10 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -352,6 +364,4287 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA32E4AB-18F3-4BB4-AF4F-4B3B28085FDA}">
+  <dimension ref="A1:K529"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0.02</v>
+      </c>
+      <c r="B2">
+        <v>12007.66</v>
+      </c>
+      <c r="F2" s="5">
+        <v>140</v>
+      </c>
+      <c r="G2" s="5">
+        <v>2.0778999999999996</v>
+      </c>
+      <c r="H2">
+        <v>1.9239999999999999</v>
+      </c>
+      <c r="I2">
+        <v>66145483933.418732</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>0.03</v>
+      </c>
+      <c r="B3">
+        <v>11967</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0.05</v>
+      </c>
+      <c r="B4">
+        <v>12008.17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="B5">
+        <v>12034.15</v>
+      </c>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>0.08</v>
+      </c>
+      <c r="B6">
+        <v>11992.21</v>
+      </c>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>0.1</v>
+      </c>
+      <c r="B7">
+        <v>11947.87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>0.12</v>
+      </c>
+      <c r="B8">
+        <v>11974.44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>0.13</v>
+      </c>
+      <c r="B9">
+        <v>11997.88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>0.15</v>
+      </c>
+      <c r="B10">
+        <v>11973.03</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>0.17</v>
+      </c>
+      <c r="B11">
+        <v>11963.77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>0.19</v>
+      </c>
+      <c r="B12">
+        <v>11976.52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>0.2</v>
+      </c>
+      <c r="B13">
+        <v>11974.99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>0.22</v>
+      </c>
+      <c r="B14">
+        <v>11976.19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>0.24</v>
+      </c>
+      <c r="B15">
+        <v>12054.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>0.25</v>
+      </c>
+      <c r="B16">
+        <v>12051.64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>0.27</v>
+      </c>
+      <c r="B17">
+        <v>11999.39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="B18">
+        <v>11990.81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>0.3</v>
+      </c>
+      <c r="B19">
+        <v>11938.17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>0.32</v>
+      </c>
+      <c r="B20">
+        <v>11968.85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>0.34</v>
+      </c>
+      <c r="B21">
+        <v>11975.49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>0.35</v>
+      </c>
+      <c r="B22">
+        <v>11963.95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>0.37</v>
+      </c>
+      <c r="B23">
+        <v>11955.77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>0.39</v>
+      </c>
+      <c r="B24">
+        <v>11963.1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>0.4</v>
+      </c>
+      <c r="B25">
+        <v>11953.6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>0.42</v>
+      </c>
+      <c r="B26">
+        <v>12001.91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>0.44</v>
+      </c>
+      <c r="B27">
+        <v>11999.66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>0.45</v>
+      </c>
+      <c r="B28">
+        <v>11967.71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>0.47</v>
+      </c>
+      <c r="B29">
+        <v>11965.99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>0.49</v>
+      </c>
+      <c r="B30">
+        <v>11908.06</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>0.51</v>
+      </c>
+      <c r="B31">
+        <v>11920.94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>0.52</v>
+      </c>
+      <c r="B32">
+        <v>11921.24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>0.54</v>
+      </c>
+      <c r="B33">
+        <v>11900.85</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="B34">
+        <v>11837.83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="B35">
+        <v>11855.54</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>0.59</v>
+      </c>
+      <c r="B36">
+        <v>11857.18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>0.61</v>
+      </c>
+      <c r="B37">
+        <v>11890.36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>0.62</v>
+      </c>
+      <c r="B38">
+        <v>11897.83</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>0.64</v>
+      </c>
+      <c r="B39">
+        <v>11923.28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>0.66</v>
+      </c>
+      <c r="B40">
+        <v>11882.24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>0.67</v>
+      </c>
+      <c r="B41">
+        <v>11873.1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>0.69</v>
+      </c>
+      <c r="B42">
+        <v>11852.81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>0.71</v>
+      </c>
+      <c r="B43">
+        <v>11856.78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>0.72</v>
+      </c>
+      <c r="B44">
+        <v>11860.99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>0.74</v>
+      </c>
+      <c r="B45">
+        <v>11868.68</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>0.76</v>
+      </c>
+      <c r="B46">
+        <v>11870.82</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>0.78</v>
+      </c>
+      <c r="B47">
+        <v>11891.97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>0.79</v>
+      </c>
+      <c r="B48">
+        <v>11854.34</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>0.81</v>
+      </c>
+      <c r="B49">
+        <v>11822.81</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>0.83</v>
+      </c>
+      <c r="B50">
+        <v>11826.58</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>0.84</v>
+      </c>
+      <c r="B51">
+        <v>11774.41</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>0.86</v>
+      </c>
+      <c r="B52">
+        <v>11798.45</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>0.88</v>
+      </c>
+      <c r="B53">
+        <v>11819.04</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>0.89</v>
+      </c>
+      <c r="B54">
+        <v>11805.88</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>0.91</v>
+      </c>
+      <c r="B55">
+        <v>11748.57</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>0.93</v>
+      </c>
+      <c r="B56">
+        <v>11747.4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>0.94</v>
+      </c>
+      <c r="B57">
+        <v>11710.17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>0.96</v>
+      </c>
+      <c r="B58">
+        <v>11728.62</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>0.98</v>
+      </c>
+      <c r="B59">
+        <v>11716.4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>0.99</v>
+      </c>
+      <c r="B60">
+        <v>11713.86</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>1.01</v>
+      </c>
+      <c r="B61">
+        <v>11697.44</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>1.03</v>
+      </c>
+      <c r="B62">
+        <v>11691.03</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>1.04</v>
+      </c>
+      <c r="B63">
+        <v>11696.68</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>1.06</v>
+      </c>
+      <c r="B64">
+        <v>11717.27</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>1.08</v>
+      </c>
+      <c r="B65">
+        <v>11696.98</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B66">
+        <v>11701.9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="B67">
+        <v>11718.6</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="B68">
+        <v>11740.69</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="B69">
+        <v>11714.69</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="B70">
+        <v>11721.56</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>1.18</v>
+      </c>
+      <c r="B71">
+        <v>11735.03</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>1.2</v>
+      </c>
+      <c r="B72">
+        <v>11709.97</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>1.21</v>
+      </c>
+      <c r="B73">
+        <v>11718.02</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>1.23</v>
+      </c>
+      <c r="B74">
+        <v>11724.17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>1.25</v>
+      </c>
+      <c r="B75">
+        <v>11742</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>1.26</v>
+      </c>
+      <c r="B76">
+        <v>11760.51</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>1.28</v>
+      </c>
+      <c r="B77">
+        <v>11712.29</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>1.3</v>
+      </c>
+      <c r="B78">
+        <v>11688.23</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>1.31</v>
+      </c>
+      <c r="B79">
+        <v>11673.66</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>1.33</v>
+      </c>
+      <c r="B80">
+        <v>11670.48</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>1.35</v>
+      </c>
+      <c r="B81">
+        <v>11660.65</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>1.36</v>
+      </c>
+      <c r="B82">
+        <v>11644.98</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>1.38</v>
+      </c>
+      <c r="B83">
+        <v>11660.15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>1.4</v>
+      </c>
+      <c r="B84">
+        <v>11675.21</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>1.42</v>
+      </c>
+      <c r="B85">
+        <v>11647.68</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>1.43</v>
+      </c>
+      <c r="B86">
+        <v>11639.49</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>1.45</v>
+      </c>
+      <c r="B87">
+        <v>11622.85</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>1.47</v>
+      </c>
+      <c r="B88">
+        <v>11580.09</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>1.48</v>
+      </c>
+      <c r="B89">
+        <v>11584.85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>1.5</v>
+      </c>
+      <c r="B90">
+        <v>11605.55</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>1.52</v>
+      </c>
+      <c r="B91">
+        <v>11618.61</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>1.53</v>
+      </c>
+      <c r="B92">
+        <v>11610.25</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>1.55</v>
+      </c>
+      <c r="B93">
+        <v>11548.08</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>1.57</v>
+      </c>
+      <c r="B94">
+        <v>11538.9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>1.58</v>
+      </c>
+      <c r="B95">
+        <v>11573.93</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>1.6</v>
+      </c>
+      <c r="B96">
+        <v>11604.61</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>1.62</v>
+      </c>
+      <c r="B97">
+        <v>11562.04</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>1.63</v>
+      </c>
+      <c r="B98">
+        <v>11554.32</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>1.65</v>
+      </c>
+      <c r="B99">
+        <v>11580.96</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>1.67</v>
+      </c>
+      <c r="B100">
+        <v>11582.94</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>1.69</v>
+      </c>
+      <c r="B101">
+        <v>11605.92</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>1.7</v>
+      </c>
+      <c r="B102">
+        <v>11594.68</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>1.72</v>
+      </c>
+      <c r="B103">
+        <v>11593.04</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>1.74</v>
+      </c>
+      <c r="B104">
+        <v>11588.51</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>1.75</v>
+      </c>
+      <c r="B105">
+        <v>11582.52</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>1.77</v>
+      </c>
+      <c r="B106">
+        <v>11553.18</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>1.79</v>
+      </c>
+      <c r="B107">
+        <v>11606.95</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>1.8</v>
+      </c>
+      <c r="B108">
+        <v>11602.54</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>1.82</v>
+      </c>
+      <c r="B109">
+        <v>11574.43</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>1.84</v>
+      </c>
+      <c r="B110">
+        <v>11634.68</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>1.85</v>
+      </c>
+      <c r="B111">
+        <v>11603.82</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>1.87</v>
+      </c>
+      <c r="B112">
+        <v>11604.33</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>1.89</v>
+      </c>
+      <c r="B113">
+        <v>11613.3</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>1.9</v>
+      </c>
+      <c r="B114">
+        <v>11632.02</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>1.92</v>
+      </c>
+      <c r="B115">
+        <v>11599.55</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>1.94</v>
+      </c>
+      <c r="B116">
+        <v>11576.71</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>1.95</v>
+      </c>
+      <c r="B117">
+        <v>11600.04</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>1.97</v>
+      </c>
+      <c r="B118">
+        <v>11544.66</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>1.99</v>
+      </c>
+      <c r="B119">
+        <v>11502.06</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="B120">
+        <v>11489.37</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>2.02</v>
+      </c>
+      <c r="B121">
+        <v>11473.48</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>2.04</v>
+      </c>
+      <c r="B122">
+        <v>11508.81</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>2.06</v>
+      </c>
+      <c r="B123">
+        <v>11491.98</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="B124">
+        <v>11468.17</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>2.09</v>
+      </c>
+      <c r="B125">
+        <v>11499.71</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>2.11</v>
+      </c>
+      <c r="B126">
+        <v>11483.05</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>2.12</v>
+      </c>
+      <c r="B127">
+        <v>11477.97</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>2.14</v>
+      </c>
+      <c r="B128">
+        <v>11467.64</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>2.16</v>
+      </c>
+      <c r="B129">
+        <v>11446.74</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>2.17</v>
+      </c>
+      <c r="B130">
+        <v>11462.08</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>2.19</v>
+      </c>
+      <c r="B131">
+        <v>11505.14</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>2.21</v>
+      </c>
+      <c r="B132">
+        <v>11459.72</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="B133">
+        <v>11483.79</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="B134">
+        <v>11500.52</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="B135">
+        <v>11476.53</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>2.2799999999999998</v>
+      </c>
+      <c r="B136">
+        <v>11502.81</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>2.29</v>
+      </c>
+      <c r="B137">
+        <v>11479.13</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>2.31</v>
+      </c>
+      <c r="B138">
+        <v>11511.71</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>2.33</v>
+      </c>
+      <c r="B139">
+        <v>11551.76</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>2.34</v>
+      </c>
+      <c r="B140">
+        <v>11480.4</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>2.36</v>
+      </c>
+      <c r="B141">
+        <v>11421.91</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>2.38</v>
+      </c>
+      <c r="B142">
+        <v>11424.56</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>2.39</v>
+      </c>
+      <c r="B143">
+        <v>11418.82</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>2.41</v>
+      </c>
+      <c r="B144">
+        <v>11416.36</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="B145">
+        <v>11466.99</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>2.44</v>
+      </c>
+      <c r="B146">
+        <v>11448.81</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>2.46</v>
+      </c>
+      <c r="B147">
+        <v>11442.01</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>2.48</v>
+      </c>
+      <c r="B148">
+        <v>11433.85</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="B149">
+        <v>11405.94</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="B150">
+        <v>11280.18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>2.5299999999999998</v>
+      </c>
+      <c r="B151">
+        <v>10730.47</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>2.54</v>
+      </c>
+      <c r="B152">
+        <v>9909.18</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>2.56</v>
+      </c>
+      <c r="B153">
+        <v>9091.4</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>2.58</v>
+      </c>
+      <c r="B154">
+        <v>8290.23</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>2.6</v>
+      </c>
+      <c r="B155">
+        <v>7580.58</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>2.61</v>
+      </c>
+      <c r="B156">
+        <v>6919.27</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>2.63</v>
+      </c>
+      <c r="B157">
+        <v>6374.53</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>2.65</v>
+      </c>
+      <c r="B158">
+        <v>5925.79</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>2.66</v>
+      </c>
+      <c r="B159">
+        <v>5543.84</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>2.68</v>
+      </c>
+      <c r="B160">
+        <v>5216.29</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>2.7</v>
+      </c>
+      <c r="B161">
+        <v>4957.46</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>2.71</v>
+      </c>
+      <c r="B162">
+        <v>4757.74</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>2.73</v>
+      </c>
+      <c r="B163">
+        <v>4586.87</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>2.75</v>
+      </c>
+      <c r="B164">
+        <v>4478.26</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>2.76</v>
+      </c>
+      <c r="B165">
+        <v>4411.3500000000004</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>2.78</v>
+      </c>
+      <c r="B166">
+        <v>4332.07</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>2.8</v>
+      </c>
+      <c r="B167">
+        <v>4321.28</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>2.81</v>
+      </c>
+      <c r="B168">
+        <v>4338.63</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>2.83</v>
+      </c>
+      <c r="B169">
+        <v>4344.0600000000004</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>2.85</v>
+      </c>
+      <c r="B170">
+        <v>4410.2</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>2.86</v>
+      </c>
+      <c r="B171">
+        <v>4490.91</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>2.88</v>
+      </c>
+      <c r="B172">
+        <v>4613.7</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>2.9</v>
+      </c>
+      <c r="B173">
+        <v>4719.87</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>2.92</v>
+      </c>
+      <c r="B174">
+        <v>4862.07</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>2.93</v>
+      </c>
+      <c r="B175">
+        <v>5011.12</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>2.95</v>
+      </c>
+      <c r="B176">
+        <v>5158.08</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>2.97</v>
+      </c>
+      <c r="B177">
+        <v>5316.14</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>2.98</v>
+      </c>
+      <c r="B178">
+        <v>5480.93</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>3</v>
+      </c>
+      <c r="B179">
+        <v>5653.86</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>3.02</v>
+      </c>
+      <c r="B180">
+        <v>5876.45</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>3.03</v>
+      </c>
+      <c r="B181">
+        <v>6048.68</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>3.05</v>
+      </c>
+      <c r="B182">
+        <v>6248.78</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>3.07</v>
+      </c>
+      <c r="B183">
+        <v>6427</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>3.08</v>
+      </c>
+      <c r="B184">
+        <v>6674.77</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>3.1</v>
+      </c>
+      <c r="B185">
+        <v>6892.98</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>3.12</v>
+      </c>
+      <c r="B186">
+        <v>7020.75</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>3.13</v>
+      </c>
+      <c r="B187">
+        <v>7226.25</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>3.15</v>
+      </c>
+      <c r="B188">
+        <v>7408.4</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>3.17</v>
+      </c>
+      <c r="B189">
+        <v>7599.71</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>3.19</v>
+      </c>
+      <c r="B190">
+        <v>7788.63</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>3.2</v>
+      </c>
+      <c r="B191">
+        <v>8009.24</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>3.22</v>
+      </c>
+      <c r="B192">
+        <v>8131.39</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>3.24</v>
+      </c>
+      <c r="B193">
+        <v>8274.9599999999991</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>3.25</v>
+      </c>
+      <c r="B194">
+        <v>8416.5499999999993</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>3.27</v>
+      </c>
+      <c r="B195">
+        <v>8545.7900000000009</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>3.29</v>
+      </c>
+      <c r="B196">
+        <v>8640.9</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>3.3</v>
+      </c>
+      <c r="B197">
+        <v>8741.77</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>3.32</v>
+      </c>
+      <c r="B198">
+        <v>8929.3799999999992</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>3.34</v>
+      </c>
+      <c r="B199">
+        <v>8999.49</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>3.35</v>
+      </c>
+      <c r="B200">
+        <v>9163.57</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>3.37</v>
+      </c>
+      <c r="B201">
+        <v>9261.9500000000007</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>3.39</v>
+      </c>
+      <c r="B202">
+        <v>9335.1</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>3.4</v>
+      </c>
+      <c r="B203">
+        <v>9425.1200000000008</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>3.42</v>
+      </c>
+      <c r="B204">
+        <v>9524.9</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>3.44</v>
+      </c>
+      <c r="B205">
+        <v>9566.86</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>3.45</v>
+      </c>
+      <c r="B206">
+        <v>9685.01</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>3.47</v>
+      </c>
+      <c r="B207">
+        <v>9767.7099999999991</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>3.49</v>
+      </c>
+      <c r="B208">
+        <v>9798.48</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>3.51</v>
+      </c>
+      <c r="B209">
+        <v>9857.51</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>3.52</v>
+      </c>
+      <c r="B210">
+        <v>9889.7999999999993</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>3.54</v>
+      </c>
+      <c r="B211">
+        <v>9979.14</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>3.56</v>
+      </c>
+      <c r="B212">
+        <v>9998.2999999999993</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>3.57</v>
+      </c>
+      <c r="B213">
+        <v>10063.84</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>3.59</v>
+      </c>
+      <c r="B214">
+        <v>10117.719999999999</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>3.61</v>
+      </c>
+      <c r="B215">
+        <v>10214.17</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>3.62</v>
+      </c>
+      <c r="B216">
+        <v>10196.35</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>3.64</v>
+      </c>
+      <c r="B217">
+        <v>10250.879999999999</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>3.66</v>
+      </c>
+      <c r="B218">
+        <v>10273.290000000001</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>3.67</v>
+      </c>
+      <c r="B219">
+        <v>10350.879999999999</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>3.69</v>
+      </c>
+      <c r="B220">
+        <v>10343.27</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>3.71</v>
+      </c>
+      <c r="B221">
+        <v>10328.19</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>3.72</v>
+      </c>
+      <c r="B222">
+        <v>10392.76</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>3.74</v>
+      </c>
+      <c r="B223">
+        <v>10406.049999999999</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>3.76</v>
+      </c>
+      <c r="B224">
+        <v>10420.74</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>3.77</v>
+      </c>
+      <c r="B225">
+        <v>10457.969999999999</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>3.79</v>
+      </c>
+      <c r="B226">
+        <v>10521.14</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>3.81</v>
+      </c>
+      <c r="B227">
+        <v>10551.29</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>3.83</v>
+      </c>
+      <c r="B228">
+        <v>10573.91</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>3.84</v>
+      </c>
+      <c r="B229">
+        <v>10584.79</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>3.86</v>
+      </c>
+      <c r="B230">
+        <v>10626.74</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>3.88</v>
+      </c>
+      <c r="B231">
+        <v>10614.12</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>3.89</v>
+      </c>
+      <c r="B232">
+        <v>10584.49</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>3.91</v>
+      </c>
+      <c r="B233">
+        <v>10576.81</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>3.93</v>
+      </c>
+      <c r="B234">
+        <v>10566.99</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>3.94</v>
+      </c>
+      <c r="B235">
+        <v>10586.26</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>3.96</v>
+      </c>
+      <c r="B236">
+        <v>10651.33</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>3.98</v>
+      </c>
+      <c r="B237">
+        <v>10656.33</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>3.99</v>
+      </c>
+      <c r="B238">
+        <v>10694.61</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>4.01</v>
+      </c>
+      <c r="B239">
+        <v>10709.56</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A240">
+        <v>4.03</v>
+      </c>
+      <c r="B240">
+        <v>10722.15</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>4.04</v>
+      </c>
+      <c r="B241">
+        <v>10750.97</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>4.0599999999999996</v>
+      </c>
+      <c r="B242">
+        <v>10781.22</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>4.08</v>
+      </c>
+      <c r="B243">
+        <v>10781.92</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B244">
+        <v>10792.18</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="B245">
+        <v>10724.84</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>4.13</v>
+      </c>
+      <c r="B246">
+        <v>10734.37</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="B247">
+        <v>10752.25</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>4.16</v>
+      </c>
+      <c r="B248">
+        <v>10737.34</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>4.18</v>
+      </c>
+      <c r="B249">
+        <v>10790.56</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>4.2</v>
+      </c>
+      <c r="B250">
+        <v>10828.91</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>4.21</v>
+      </c>
+      <c r="B251">
+        <v>10816.16</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="B252">
+        <v>10825.44</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A253">
+        <v>4.25</v>
+      </c>
+      <c r="B253">
+        <v>10811.17</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A254">
+        <v>4.26</v>
+      </c>
+      <c r="B254">
+        <v>10823.01</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A255">
+        <v>4.28</v>
+      </c>
+      <c r="B255">
+        <v>10812.98</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A256">
+        <v>4.3</v>
+      </c>
+      <c r="B256">
+        <v>10817.75</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A257">
+        <v>4.3099999999999996</v>
+      </c>
+      <c r="B257">
+        <v>10810.52</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A258">
+        <v>4.33</v>
+      </c>
+      <c r="B258">
+        <v>10791.81</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A259">
+        <v>4.3499999999999996</v>
+      </c>
+      <c r="B259">
+        <v>10831.38</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A260">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="B260">
+        <v>10834.55</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A261">
+        <v>4.38</v>
+      </c>
+      <c r="B261">
+        <v>10798.92</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A262">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="B262">
+        <v>10827.02</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A263">
+        <v>4.42</v>
+      </c>
+      <c r="B263">
+        <v>10806.12</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A264">
+        <v>4.43</v>
+      </c>
+      <c r="B264">
+        <v>10828.5</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A265">
+        <v>4.45</v>
+      </c>
+      <c r="B265">
+        <v>10821.5</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A266">
+        <v>4.47</v>
+      </c>
+      <c r="B266">
+        <v>10845.18</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A267">
+        <v>4.4800000000000004</v>
+      </c>
+      <c r="B267">
+        <v>10845.5</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A268">
+        <v>4.5</v>
+      </c>
+      <c r="B268">
+        <v>10789.69</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A269">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="B269">
+        <v>10795.28</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A270">
+        <v>4.53</v>
+      </c>
+      <c r="B270">
+        <v>10787.63</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A271">
+        <v>4.55</v>
+      </c>
+      <c r="B271">
+        <v>10792.65</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A272">
+        <v>4.57</v>
+      </c>
+      <c r="B272">
+        <v>10789.15</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A273">
+        <v>4.58</v>
+      </c>
+      <c r="B273">
+        <v>10783.32</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A274">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="B274">
+        <v>10787.46</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A275">
+        <v>4.62</v>
+      </c>
+      <c r="B275">
+        <v>10817.82</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A276">
+        <v>4.63</v>
+      </c>
+      <c r="B276">
+        <v>10790.14</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A277">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="B277">
+        <v>10747.12</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A278">
+        <v>4.67</v>
+      </c>
+      <c r="B278">
+        <v>10816.35</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A279">
+        <v>4.68</v>
+      </c>
+      <c r="B279">
+        <v>10796.93</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A280">
+        <v>4.7</v>
+      </c>
+      <c r="B280">
+        <v>10808.11</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A281">
+        <v>4.72</v>
+      </c>
+      <c r="B281">
+        <v>10829.37</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A282">
+        <v>4.74</v>
+      </c>
+      <c r="B282">
+        <v>10877.45</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A283">
+        <v>4.75</v>
+      </c>
+      <c r="B283">
+        <v>10849.25</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A284">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="B284">
+        <v>10854.6</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A285">
+        <v>4.79</v>
+      </c>
+      <c r="B285">
+        <v>10837.45</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A286">
+        <v>4.8</v>
+      </c>
+      <c r="B286">
+        <v>10830.93</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A287">
+        <v>4.82</v>
+      </c>
+      <c r="B287">
+        <v>10852.07</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A288">
+        <v>4.84</v>
+      </c>
+      <c r="B288">
+        <v>11296.65</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A289">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="B289">
+        <v>12264.86</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>4.87</v>
+      </c>
+      <c r="B290">
+        <v>13303.34</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A291">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="B291">
+        <v>14283.42</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A292">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="B292">
+        <v>15036.93</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A293">
+        <v>4.92</v>
+      </c>
+      <c r="B293">
+        <v>15624.52</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A294">
+        <v>4.9400000000000004</v>
+      </c>
+      <c r="B294">
+        <v>16016.7</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A295">
+        <v>4.95</v>
+      </c>
+      <c r="B295">
+        <v>16312.52</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A296">
+        <v>4.97</v>
+      </c>
+      <c r="B296">
+        <v>16554.39</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A297">
+        <v>4.99</v>
+      </c>
+      <c r="B297">
+        <v>16669.599999999999</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A298">
+        <v>5.01</v>
+      </c>
+      <c r="B298">
+        <v>16695.990000000002</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A299">
+        <v>5.0199999999999996</v>
+      </c>
+      <c r="B299">
+        <v>16677.759999999998</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A300">
+        <v>5.04</v>
+      </c>
+      <c r="B300">
+        <v>16731.66</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A301">
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="B301">
+        <v>16646.04</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>5.07</v>
+      </c>
+      <c r="B302">
+        <v>16522.900000000001</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A303">
+        <v>5.09</v>
+      </c>
+      <c r="B303">
+        <v>16392.400000000001</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>5.1100000000000003</v>
+      </c>
+      <c r="B304">
+        <v>16339.63</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>5.12</v>
+      </c>
+      <c r="B305">
+        <v>16232.96</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A306">
+        <v>5.14</v>
+      </c>
+      <c r="B306">
+        <v>16044.17</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>5.16</v>
+      </c>
+      <c r="B307">
+        <v>15874.42</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A308">
+        <v>5.17</v>
+      </c>
+      <c r="B308">
+        <v>15777.69</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>5.19</v>
+      </c>
+      <c r="B309">
+        <v>15575.33</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>5.21</v>
+      </c>
+      <c r="B310">
+        <v>15501.73</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>5.22</v>
+      </c>
+      <c r="B311">
+        <v>15349.4</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>5.24</v>
+      </c>
+      <c r="B312">
+        <v>15237.31</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>5.26</v>
+      </c>
+      <c r="B313">
+        <v>15105.07</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>5.27</v>
+      </c>
+      <c r="B314">
+        <v>14966.17</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A315">
+        <v>5.29</v>
+      </c>
+      <c r="B315">
+        <v>14806.55</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A316">
+        <v>5.31</v>
+      </c>
+      <c r="B316">
+        <v>14728.22</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A317">
+        <v>5.33</v>
+      </c>
+      <c r="B317">
+        <v>14560.08</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A318">
+        <v>5.34</v>
+      </c>
+      <c r="B318">
+        <v>14457</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A319">
+        <v>5.36</v>
+      </c>
+      <c r="B319">
+        <v>14290.93</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A320">
+        <v>5.38</v>
+      </c>
+      <c r="B320">
+        <v>14155.29</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A321">
+        <v>5.39</v>
+      </c>
+      <c r="B321">
+        <v>14060.55</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A322">
+        <v>5.41</v>
+      </c>
+      <c r="B322">
+        <v>14015.86</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A323">
+        <v>5.43</v>
+      </c>
+      <c r="B323">
+        <v>13955.04</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A324">
+        <v>5.44</v>
+      </c>
+      <c r="B324">
+        <v>13856.74</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A325">
+        <v>5.46</v>
+      </c>
+      <c r="B325">
+        <v>13798.45</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A326">
+        <v>5.48</v>
+      </c>
+      <c r="B326">
+        <v>13659.75</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A327">
+        <v>5.49</v>
+      </c>
+      <c r="B327">
+        <v>13630.86</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A328">
+        <v>5.51</v>
+      </c>
+      <c r="B328">
+        <v>13545.01</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A329">
+        <v>5.53</v>
+      </c>
+      <c r="B329">
+        <v>13469.54</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A330">
+        <v>5.54</v>
+      </c>
+      <c r="B330">
+        <v>13382.92</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A331">
+        <v>5.56</v>
+      </c>
+      <c r="B331">
+        <v>13250.67</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>5.58</v>
+      </c>
+      <c r="B332">
+        <v>13193.34</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>5.59</v>
+      </c>
+      <c r="B333">
+        <v>13106.41</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>5.61</v>
+      </c>
+      <c r="B334">
+        <v>13014.22</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>5.63</v>
+      </c>
+      <c r="B335">
+        <v>13002.51</v>
+      </c>
+    </row>
+    <row r="336" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>5.65</v>
+      </c>
+      <c r="B336">
+        <v>12987.67</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>5.66</v>
+      </c>
+      <c r="B337">
+        <v>12906.23</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>5.68</v>
+      </c>
+      <c r="B338">
+        <v>12794.27</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>5.7</v>
+      </c>
+      <c r="B339">
+        <v>12712.1</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>5.71</v>
+      </c>
+      <c r="B340">
+        <v>12659.73</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A341">
+        <v>5.73</v>
+      </c>
+      <c r="B341">
+        <v>12613.45</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A342">
+        <v>5.75</v>
+      </c>
+      <c r="B342">
+        <v>12542.73</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>5.76</v>
+      </c>
+      <c r="B343">
+        <v>12467.22</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>5.78</v>
+      </c>
+      <c r="B344">
+        <v>12472.88</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A345">
+        <v>5.8</v>
+      </c>
+      <c r="B345">
+        <v>12463.35</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A346">
+        <v>5.81</v>
+      </c>
+      <c r="B346">
+        <v>12424.68</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A347">
+        <v>5.83</v>
+      </c>
+      <c r="B347">
+        <v>12381.43</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A348">
+        <v>5.85</v>
+      </c>
+      <c r="B348">
+        <v>12377.05</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A349">
+        <v>5.86</v>
+      </c>
+      <c r="B349">
+        <v>12319.64</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A350">
+        <v>5.88</v>
+      </c>
+      <c r="B350">
+        <v>12193.92</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A351">
+        <v>5.9</v>
+      </c>
+      <c r="B351">
+        <v>12191.04</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A352">
+        <v>5.92</v>
+      </c>
+      <c r="B352">
+        <v>12154.44</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A353">
+        <v>5.93</v>
+      </c>
+      <c r="B353">
+        <v>12100.9</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A354">
+        <v>5.95</v>
+      </c>
+      <c r="B354">
+        <v>12090.74</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A355">
+        <v>5.97</v>
+      </c>
+      <c r="B355">
+        <v>12046.47</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A356">
+        <v>5.98</v>
+      </c>
+      <c r="B356">
+        <v>12047.01</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A357">
+        <v>6</v>
+      </c>
+      <c r="B357">
+        <v>12031.1</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A358">
+        <v>6.02</v>
+      </c>
+      <c r="B358">
+        <v>12024.57</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A359">
+        <v>6.03</v>
+      </c>
+      <c r="B359">
+        <v>11933.22</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A360">
+        <v>6.05</v>
+      </c>
+      <c r="B360">
+        <v>11961.77</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A361">
+        <v>6.07</v>
+      </c>
+      <c r="B361">
+        <v>11877.03</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A362">
+        <v>6.08</v>
+      </c>
+      <c r="B362">
+        <v>11834.65</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A363">
+        <v>6.1</v>
+      </c>
+      <c r="B363">
+        <v>11864.54</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A364">
+        <v>6.12</v>
+      </c>
+      <c r="B364">
+        <v>11823.32</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A365">
+        <v>6.13</v>
+      </c>
+      <c r="B365">
+        <v>11767.42</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A366">
+        <v>6.15</v>
+      </c>
+      <c r="B366">
+        <v>11734.14</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A367">
+        <v>6.17</v>
+      </c>
+      <c r="B367">
+        <v>11645.09</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A368">
+        <v>6.18</v>
+      </c>
+      <c r="B368">
+        <v>11600.73</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A369">
+        <v>6.2</v>
+      </c>
+      <c r="B369">
+        <v>11665.45</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A370">
+        <v>6.22</v>
+      </c>
+      <c r="B370">
+        <v>11628.74</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A371">
+        <v>6.24</v>
+      </c>
+      <c r="B371">
+        <v>11634.19</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A372">
+        <v>6.25</v>
+      </c>
+      <c r="B372">
+        <v>11609.82</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A373">
+        <v>6.27</v>
+      </c>
+      <c r="B373">
+        <v>11602.29</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A374">
+        <v>6.29</v>
+      </c>
+      <c r="B374">
+        <v>11559.69</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>6.3</v>
+      </c>
+      <c r="B375">
+        <v>11573.19</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>6.32</v>
+      </c>
+      <c r="B376">
+        <v>11532.42</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A377">
+        <v>6.34</v>
+      </c>
+      <c r="B377">
+        <v>11495.61</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A378">
+        <v>6.35</v>
+      </c>
+      <c r="B378">
+        <v>11519.05</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A379">
+        <v>6.37</v>
+      </c>
+      <c r="B379">
+        <v>11495.43</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A380">
+        <v>6.39</v>
+      </c>
+      <c r="B380">
+        <v>11461.52</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A381">
+        <v>6.4</v>
+      </c>
+      <c r="B381">
+        <v>11443.33</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A382">
+        <v>6.42</v>
+      </c>
+      <c r="B382">
+        <v>11439.27</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A383">
+        <v>6.44</v>
+      </c>
+      <c r="B383">
+        <v>11446.06</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A384">
+        <v>6.45</v>
+      </c>
+      <c r="B384">
+        <v>11472.01</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A385">
+        <v>6.47</v>
+      </c>
+      <c r="B385">
+        <v>11514.57</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A386">
+        <v>6.49</v>
+      </c>
+      <c r="B386">
+        <v>11490.86</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A387">
+        <v>6.5</v>
+      </c>
+      <c r="B387">
+        <v>11445.05</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A388">
+        <v>6.52</v>
+      </c>
+      <c r="B388">
+        <v>11418.72</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A389">
+        <v>6.54</v>
+      </c>
+      <c r="B389">
+        <v>11337.32</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A390">
+        <v>6.56</v>
+      </c>
+      <c r="B390">
+        <v>11272.03</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A391">
+        <v>6.57</v>
+      </c>
+      <c r="B391">
+        <v>11308.36</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A392">
+        <v>6.59</v>
+      </c>
+      <c r="B392">
+        <v>11297.27</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A393">
+        <v>6.61</v>
+      </c>
+      <c r="B393">
+        <v>11295.46</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A394">
+        <v>6.62</v>
+      </c>
+      <c r="B394">
+        <v>11264.25</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A395">
+        <v>6.64</v>
+      </c>
+      <c r="B395">
+        <v>11217.09</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A396">
+        <v>6.66</v>
+      </c>
+      <c r="B396">
+        <v>11230.64</v>
+      </c>
+    </row>
+    <row r="397" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A397">
+        <v>6.67</v>
+      </c>
+      <c r="B397">
+        <v>11231.12</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A398">
+        <v>6.69</v>
+      </c>
+      <c r="B398">
+        <v>11288.43</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A399">
+        <v>6.71</v>
+      </c>
+      <c r="B399">
+        <v>11256.58</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A400">
+        <v>6.72</v>
+      </c>
+      <c r="B400">
+        <v>11214.96</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A401">
+        <v>6.74</v>
+      </c>
+      <c r="B401">
+        <v>11190.25</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A402">
+        <v>6.76</v>
+      </c>
+      <c r="B402">
+        <v>11217.63</v>
+      </c>
+    </row>
+    <row r="403" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A403">
+        <v>6.77</v>
+      </c>
+      <c r="B403">
+        <v>11174.85</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A404">
+        <v>6.79</v>
+      </c>
+      <c r="B404">
+        <v>11234.41</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A405">
+        <v>6.81</v>
+      </c>
+      <c r="B405">
+        <v>11198.18</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A406">
+        <v>6.83</v>
+      </c>
+      <c r="B406">
+        <v>11152.67</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A407">
+        <v>6.84</v>
+      </c>
+      <c r="B407">
+        <v>11175.52</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A408">
+        <v>6.86</v>
+      </c>
+      <c r="B408">
+        <v>11187.48</v>
+      </c>
+    </row>
+    <row r="409" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A409">
+        <v>6.88</v>
+      </c>
+      <c r="B409">
+        <v>11169.49</v>
+      </c>
+    </row>
+    <row r="410" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A410">
+        <v>6.89</v>
+      </c>
+      <c r="B410">
+        <v>11113.89</v>
+      </c>
+    </row>
+    <row r="411" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A411">
+        <v>6.91</v>
+      </c>
+      <c r="B411">
+        <v>11098.24</v>
+      </c>
+    </row>
+    <row r="412" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A412">
+        <v>6.93</v>
+      </c>
+      <c r="B412">
+        <v>11075.6</v>
+      </c>
+    </row>
+    <row r="413" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A413">
+        <v>6.94</v>
+      </c>
+      <c r="B413">
+        <v>11121.79</v>
+      </c>
+    </row>
+    <row r="414" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A414">
+        <v>6.96</v>
+      </c>
+      <c r="B414">
+        <v>11074.34</v>
+      </c>
+    </row>
+    <row r="415" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A415">
+        <v>6.98</v>
+      </c>
+      <c r="B415">
+        <v>11089.79</v>
+      </c>
+    </row>
+    <row r="416" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A416">
+        <v>6.99</v>
+      </c>
+      <c r="B416">
+        <v>11022.62</v>
+      </c>
+    </row>
+    <row r="417" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A417">
+        <v>7.01</v>
+      </c>
+      <c r="B417">
+        <v>11052.36</v>
+      </c>
+    </row>
+    <row r="418" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A418">
+        <v>7.03</v>
+      </c>
+      <c r="B418">
+        <v>11041.05</v>
+      </c>
+    </row>
+    <row r="419" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A419">
+        <v>7.04</v>
+      </c>
+      <c r="B419">
+        <v>11074.67</v>
+      </c>
+    </row>
+    <row r="420" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A420">
+        <v>7.06</v>
+      </c>
+      <c r="B420">
+        <v>11022.16</v>
+      </c>
+    </row>
+    <row r="421" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A421">
+        <v>7.08</v>
+      </c>
+      <c r="B421">
+        <v>10975.81</v>
+      </c>
+    </row>
+    <row r="422" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A422">
+        <v>7.09</v>
+      </c>
+      <c r="B422">
+        <v>10976.82</v>
+      </c>
+    </row>
+    <row r="423" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A423">
+        <v>7.11</v>
+      </c>
+      <c r="B423">
+        <v>10993.48</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A424">
+        <v>7.13</v>
+      </c>
+      <c r="B424">
+        <v>10968.85</v>
+      </c>
+    </row>
+    <row r="425" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A425">
+        <v>7.15</v>
+      </c>
+      <c r="B425">
+        <v>10956.75</v>
+      </c>
+    </row>
+    <row r="426" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A426">
+        <v>7.16</v>
+      </c>
+      <c r="B426">
+        <v>10972.06</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A427">
+        <v>7.18</v>
+      </c>
+      <c r="B427">
+        <v>10958.69</v>
+      </c>
+    </row>
+    <row r="428" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A428">
+        <v>7.2</v>
+      </c>
+      <c r="B428">
+        <v>10977.45</v>
+      </c>
+    </row>
+    <row r="429" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A429">
+        <v>7.21</v>
+      </c>
+      <c r="B429">
+        <v>10949.11</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A430">
+        <v>7.23</v>
+      </c>
+      <c r="B430">
+        <v>10918.45</v>
+      </c>
+    </row>
+    <row r="431" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A431">
+        <v>7.25</v>
+      </c>
+      <c r="B431">
+        <v>10964.41</v>
+      </c>
+    </row>
+    <row r="432" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A432">
+        <v>7.26</v>
+      </c>
+      <c r="B432">
+        <v>10965.24</v>
+      </c>
+    </row>
+    <row r="433" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A433">
+        <v>7.28</v>
+      </c>
+      <c r="B433">
+        <v>10952.5</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A434">
+        <v>7.3</v>
+      </c>
+      <c r="B434">
+        <v>10979.03</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A435">
+        <v>7.31</v>
+      </c>
+      <c r="B435">
+        <v>10973.76</v>
+      </c>
+    </row>
+    <row r="436" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A436">
+        <v>7.33</v>
+      </c>
+      <c r="B436">
+        <v>10970.88</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A437">
+        <v>7.35</v>
+      </c>
+      <c r="B437">
+        <v>10972.21</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A438">
+        <v>7.36</v>
+      </c>
+      <c r="B438">
+        <v>10963.65</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A439">
+        <v>7.38</v>
+      </c>
+      <c r="B439">
+        <v>10954.82</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A440">
+        <v>7.4</v>
+      </c>
+      <c r="B440">
+        <v>10920.78</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A441">
+        <v>7.41</v>
+      </c>
+      <c r="B441">
+        <v>10885.24</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A442">
+        <v>7.43</v>
+      </c>
+      <c r="B442">
+        <v>10902.51</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A443">
+        <v>7.45</v>
+      </c>
+      <c r="B443">
+        <v>10887.76</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A444">
+        <v>7.47</v>
+      </c>
+      <c r="B444">
+        <v>10873.18</v>
+      </c>
+    </row>
+    <row r="445" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A445">
+        <v>7.48</v>
+      </c>
+      <c r="B445">
+        <v>10852.29</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A446">
+        <v>7.5</v>
+      </c>
+      <c r="B446">
+        <v>10870.53</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A447">
+        <v>7.52</v>
+      </c>
+      <c r="B447">
+        <v>10880.71</v>
+      </c>
+    </row>
+    <row r="448" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A448">
+        <v>7.53</v>
+      </c>
+      <c r="B448">
+        <v>10938.66</v>
+      </c>
+    </row>
+    <row r="449" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A449">
+        <v>7.55</v>
+      </c>
+      <c r="B449">
+        <v>10933.83</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A450">
+        <v>7.57</v>
+      </c>
+      <c r="B450">
+        <v>10926.4</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A451">
+        <v>7.58</v>
+      </c>
+      <c r="B451">
+        <v>10909.61</v>
+      </c>
+    </row>
+    <row r="452" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A452">
+        <v>7.6</v>
+      </c>
+      <c r="B452">
+        <v>10886.24</v>
+      </c>
+    </row>
+    <row r="453" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A453">
+        <v>7.62</v>
+      </c>
+      <c r="B453">
+        <v>10892.35</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A454">
+        <v>7.63</v>
+      </c>
+      <c r="B454">
+        <v>10849.24</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A455">
+        <v>7.65</v>
+      </c>
+      <c r="B455">
+        <v>10789.93</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A456">
+        <v>7.67</v>
+      </c>
+      <c r="B456">
+        <v>10822.09</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A457">
+        <v>7.68</v>
+      </c>
+      <c r="B457">
+        <v>10839.41</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A458">
+        <v>7.7</v>
+      </c>
+      <c r="B458">
+        <v>10838.3</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A459">
+        <v>7.72</v>
+      </c>
+      <c r="B459">
+        <v>10834.74</v>
+      </c>
+    </row>
+    <row r="460" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A460">
+        <v>7.74</v>
+      </c>
+      <c r="B460">
+        <v>10823.13</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A461">
+        <v>7.75</v>
+      </c>
+      <c r="B461">
+        <v>10802.49</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A462">
+        <v>7.77</v>
+      </c>
+      <c r="B462">
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A463">
+        <v>7.79</v>
+      </c>
+      <c r="B463">
+        <v>10782.84</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A464">
+        <v>7.8</v>
+      </c>
+      <c r="B464">
+        <v>10793.33</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A465">
+        <v>7.82</v>
+      </c>
+      <c r="B465">
+        <v>10830.99</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A466">
+        <v>7.84</v>
+      </c>
+      <c r="B466">
+        <v>10865.35</v>
+      </c>
+    </row>
+    <row r="467" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A467">
+        <v>7.85</v>
+      </c>
+      <c r="B467">
+        <v>10854.25</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A468">
+        <v>7.87</v>
+      </c>
+      <c r="B468">
+        <v>10827.17</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A469">
+        <v>7.89</v>
+      </c>
+      <c r="B469">
+        <v>10796.1</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A470">
+        <v>7.9</v>
+      </c>
+      <c r="B470">
+        <v>10792.94</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A471">
+        <v>7.92</v>
+      </c>
+      <c r="B471">
+        <v>10784.08</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A472">
+        <v>7.94</v>
+      </c>
+      <c r="B472">
+        <v>10748.63</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A473">
+        <v>7.95</v>
+      </c>
+      <c r="B473">
+        <v>10707.36</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A474">
+        <v>7.97</v>
+      </c>
+      <c r="B474">
+        <v>10720.19</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A475">
+        <v>7.99</v>
+      </c>
+      <c r="B475">
+        <v>10736.48</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A476">
+        <v>8</v>
+      </c>
+      <c r="B476">
+        <v>10730.65</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A477">
+        <v>8.02</v>
+      </c>
+      <c r="B477">
+        <v>10782.33</v>
+      </c>
+    </row>
+    <row r="478" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A478">
+        <v>8.0399999999999991</v>
+      </c>
+      <c r="B478">
+        <v>10788.4</v>
+      </c>
+    </row>
+    <row r="479" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A479">
+        <v>8.06</v>
+      </c>
+      <c r="B479">
+        <v>10759.75</v>
+      </c>
+    </row>
+    <row r="480" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A480">
+        <v>8.07</v>
+      </c>
+      <c r="B480">
+        <v>10757.04</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A481">
+        <v>8.09</v>
+      </c>
+      <c r="B481">
+        <v>10720.64</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A482">
+        <v>8.11</v>
+      </c>
+      <c r="B482">
+        <v>10719.53</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A483">
+        <v>8.1199999999999992</v>
+      </c>
+      <c r="B483">
+        <v>10755.34</v>
+      </c>
+    </row>
+    <row r="484" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A484">
+        <v>8.14</v>
+      </c>
+      <c r="B484">
+        <v>10701.19</v>
+      </c>
+    </row>
+    <row r="485" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A485">
+        <v>8.16</v>
+      </c>
+      <c r="B485">
+        <v>10714.03</v>
+      </c>
+    </row>
+    <row r="486" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A486">
+        <v>8.17</v>
+      </c>
+      <c r="B486">
+        <v>10703.37</v>
+      </c>
+    </row>
+    <row r="487" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A487">
+        <v>8.19</v>
+      </c>
+      <c r="B487">
+        <v>10676.28</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A488">
+        <v>8.2100000000000009</v>
+      </c>
+      <c r="B488">
+        <v>10715.35</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A489">
+        <v>8.2200000000000006</v>
+      </c>
+      <c r="B489">
+        <v>10735.72</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A490">
+        <v>8.24</v>
+      </c>
+      <c r="B490">
+        <v>10793.13</v>
+      </c>
+    </row>
+    <row r="491" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A491">
+        <v>8.26</v>
+      </c>
+      <c r="B491">
+        <v>10776.32</v>
+      </c>
+    </row>
+    <row r="492" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A492">
+        <v>8.27</v>
+      </c>
+      <c r="B492">
+        <v>10710.69</v>
+      </c>
+    </row>
+    <row r="493" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A493">
+        <v>8.2899999999999991</v>
+      </c>
+      <c r="B493">
+        <v>10733.29</v>
+      </c>
+    </row>
+    <row r="494" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A494">
+        <v>8.31</v>
+      </c>
+      <c r="B494">
+        <v>10758.28</v>
+      </c>
+    </row>
+    <row r="495" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A495">
+        <v>8.33</v>
+      </c>
+      <c r="B495">
+        <v>10755.32</v>
+      </c>
+    </row>
+    <row r="496" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A496">
+        <v>8.34</v>
+      </c>
+      <c r="B496">
+        <v>10705.73</v>
+      </c>
+    </row>
+    <row r="497" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A497">
+        <v>8.36</v>
+      </c>
+      <c r="B497">
+        <v>10721.98</v>
+      </c>
+    </row>
+    <row r="498" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A498">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="B498">
+        <v>10666.45</v>
+      </c>
+    </row>
+    <row r="499" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A499">
+        <v>8.39</v>
+      </c>
+      <c r="B499">
+        <v>10666.62</v>
+      </c>
+    </row>
+    <row r="500" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A500">
+        <v>8.41</v>
+      </c>
+      <c r="B500">
+        <v>10631.02</v>
+      </c>
+    </row>
+    <row r="501" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A501">
+        <v>8.43</v>
+      </c>
+      <c r="B501">
+        <v>10654.56</v>
+      </c>
+    </row>
+    <row r="502" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A502">
+        <v>8.44</v>
+      </c>
+      <c r="B502">
+        <v>10658.04</v>
+      </c>
+    </row>
+    <row r="503" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A503">
+        <v>8.4600000000000009</v>
+      </c>
+      <c r="B503">
+        <v>10671.23</v>
+      </c>
+    </row>
+    <row r="504" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A504">
+        <v>8.48</v>
+      </c>
+      <c r="B504">
+        <v>10710.19</v>
+      </c>
+    </row>
+    <row r="505" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A505">
+        <v>8.49</v>
+      </c>
+      <c r="B505">
+        <v>10696.69</v>
+      </c>
+    </row>
+    <row r="506" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A506">
+        <v>8.51</v>
+      </c>
+      <c r="B506">
+        <v>10704</v>
+      </c>
+    </row>
+    <row r="507" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A507">
+        <v>8.5299999999999994</v>
+      </c>
+      <c r="B507">
+        <v>10697.06</v>
+      </c>
+    </row>
+    <row r="508" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A508">
+        <v>8.5399999999999991</v>
+      </c>
+      <c r="B508">
+        <v>10669.26</v>
+      </c>
+    </row>
+    <row r="509" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A509">
+        <v>8.56</v>
+      </c>
+      <c r="B509">
+        <v>10724.5</v>
+      </c>
+    </row>
+    <row r="510" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A510">
+        <v>8.58</v>
+      </c>
+      <c r="B510">
+        <v>10713.78</v>
+      </c>
+    </row>
+    <row r="511" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A511">
+        <v>8.59</v>
+      </c>
+      <c r="B511">
+        <v>10673.04</v>
+      </c>
+    </row>
+    <row r="512" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A512">
+        <v>8.61</v>
+      </c>
+      <c r="B512">
+        <v>10683.84</v>
+      </c>
+    </row>
+    <row r="513" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A513">
+        <v>8.6300000000000008</v>
+      </c>
+      <c r="B513">
+        <v>10701.92</v>
+      </c>
+    </row>
+    <row r="514" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A514">
+        <v>8.65</v>
+      </c>
+      <c r="B514">
+        <v>10658.4</v>
+      </c>
+    </row>
+    <row r="515" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A515">
+        <v>8.66</v>
+      </c>
+      <c r="B515">
+        <v>10660.11</v>
+      </c>
+    </row>
+    <row r="516" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A516">
+        <v>8.68</v>
+      </c>
+      <c r="B516">
+        <v>10663.83</v>
+      </c>
+    </row>
+    <row r="517" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A517">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="B517">
+        <v>10684.22</v>
+      </c>
+    </row>
+    <row r="518" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A518">
+        <v>8.7100000000000009</v>
+      </c>
+      <c r="B518">
+        <v>10690.69</v>
+      </c>
+    </row>
+    <row r="519" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A519">
+        <v>8.73</v>
+      </c>
+      <c r="B519">
+        <v>10646.32</v>
+      </c>
+    </row>
+    <row r="520" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A520">
+        <v>8.75</v>
+      </c>
+      <c r="B520">
+        <v>10668.33</v>
+      </c>
+    </row>
+    <row r="521" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A521">
+        <v>8.76</v>
+      </c>
+      <c r="B521">
+        <v>10631.68</v>
+      </c>
+    </row>
+    <row r="522" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A522">
+        <v>8.7799999999999994</v>
+      </c>
+      <c r="B522">
+        <v>10625.26</v>
+      </c>
+    </row>
+    <row r="523" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A523">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="B523">
+        <v>10593.17</v>
+      </c>
+    </row>
+    <row r="524" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A524">
+        <v>8.81</v>
+      </c>
+      <c r="B524">
+        <v>10579.97</v>
+      </c>
+    </row>
+    <row r="525" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A525">
+        <v>8.83</v>
+      </c>
+      <c r="B525">
+        <v>10633.14</v>
+      </c>
+    </row>
+    <row r="526" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A526">
+        <v>8.85</v>
+      </c>
+      <c r="B526">
+        <v>10586.49</v>
+      </c>
+    </row>
+    <row r="527" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A527">
+        <v>8.86</v>
+      </c>
+      <c r="B527">
+        <v>10632.88</v>
+      </c>
+    </row>
+    <row r="528" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A528">
+        <v>8.8800000000000008</v>
+      </c>
+      <c r="B528">
+        <v>10589.14</v>
+      </c>
+    </row>
+    <row r="529" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A529">
+        <v>8.9</v>
+      </c>
+      <c r="B529">
+        <v>10631.84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF835A5-39F3-4EEB-AFA8-0C4C82D211A3}">
   <dimension ref="A1:L857"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -384,7 +4677,7 @@
       <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correction factor is now in excel, fitted parameters are now saved in scientific notation
</commit_message>
<xml_diff>
--- a/dist/example/uptake_curve.xlsx
+++ b/dist/example/uptake_curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mail\CLionProjects\0d_adsorption\dist\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4118FF5-B7E0-497E-B48B-583B0B823A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5D9923-8258-4351-84AF-D52BD5C31E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{F42F43B3-C9C7-49B5-A63B-84B6B370C241}"/>
+    <workbookView xWindow="17640" yWindow="2715" windowWidth="16770" windowHeight="15345" activeTab="1" xr2:uid="{F42F43B3-C9C7-49B5-A63B-84B6B370C241}"/>
   </bookViews>
   <sheets>
     <sheet name="levoglucosan" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
   <si>
     <t>time</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>L</t>
+  </si>
+  <si>
+    <t>Correction factor</t>
   </si>
 </sst>
 </file>
@@ -365,10 +368,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA32E4AB-18F3-4BB4-AF4F-4B3B28085FDA}">
-  <dimension ref="A1:K529"/>
+  <dimension ref="A1:L529"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="12" max="12" width="13.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -393,8 +399,11 @@
       <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="L1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.02</v>
       </c>
@@ -419,8 +428,11 @@
       <c r="K2">
         <v>40</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0.03</v>
       </c>
@@ -428,7 +440,7 @@
         <v>11967</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0.05</v>
       </c>
@@ -436,7 +448,7 @@
         <v>12008.17</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -445,7 +457,7 @@
       </c>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.08</v>
       </c>
@@ -454,7 +466,7 @@
       </c>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0.1</v>
       </c>
@@ -462,7 +474,7 @@
         <v>11947.87</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.12</v>
       </c>
@@ -470,7 +482,7 @@
         <v>11974.44</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0.13</v>
       </c>
@@ -478,7 +490,7 @@
         <v>11997.88</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0.15</v>
       </c>
@@ -486,7 +498,7 @@
         <v>11973.03</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0.17</v>
       </c>
@@ -494,7 +506,7 @@
         <v>11963.77</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0.19</v>
       </c>
@@ -502,7 +514,7 @@
         <v>11976.52</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>0.2</v>
       </c>
@@ -510,7 +522,7 @@
         <v>11974.99</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0.22</v>
       </c>
@@ -518,7 +530,7 @@
         <v>11976.19</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0.24</v>
       </c>
@@ -526,7 +538,7 @@
         <v>12054.6</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>0.25</v>
       </c>
@@ -4646,13 +4658,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF835A5-39F3-4EEB-AFA8-0C4C82D211A3}">
-  <dimension ref="A1:L857"/>
+  <dimension ref="A1:M857"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4680,8 +4693,11 @@
       <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.02</v>
       </c>
@@ -4709,8 +4725,11 @@
       <c r="L2">
         <v>1.56</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0.03</v>
       </c>
@@ -4718,7 +4737,7 @@
         <v>1214.8499999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0.05</v>
       </c>
@@ -4726,7 +4745,7 @@
         <v>1212.6300000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -4734,7 +4753,7 @@
         <v>1195.3900000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.08</v>
       </c>
@@ -4742,7 +4761,7 @@
         <v>1205.55</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0.1</v>
       </c>
@@ -4750,7 +4769,7 @@
         <v>1202.8699999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.12</v>
       </c>
@@ -4758,7 +4777,7 @@
         <v>1209.5</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0.13</v>
       </c>
@@ -4766,7 +4785,7 @@
         <v>1202.6400000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0.15</v>
       </c>
@@ -4774,7 +4793,7 @@
         <v>1202.79</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0.17</v>
       </c>
@@ -4782,7 +4801,7 @@
         <v>1199.72</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0.19</v>
       </c>
@@ -4790,7 +4809,7 @@
         <v>1191.7</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>0.2</v>
       </c>
@@ -4798,7 +4817,7 @@
         <v>1207.32</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0.22</v>
       </c>
@@ -4806,7 +4825,7 @@
         <v>1205.68</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0.24</v>
       </c>
@@ -4814,7 +4833,7 @@
         <v>1195.4000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
Created a new figure to explain the preprocessing algorithm
</commit_message>
<xml_diff>
--- a/dist/example/uptake_curve.xlsx
+++ b/dist/example/uptake_curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mail\CLionProjects\0d_adsorption\dist\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5D9923-8258-4351-84AF-D52BD5C31E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B230A0-50B3-4D3C-AEC0-0139706A2A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17640" yWindow="2715" windowWidth="16770" windowHeight="15345" activeTab="1" xr2:uid="{F42F43B3-C9C7-49B5-A63B-84B6B370C241}"/>
+    <workbookView xWindow="17640" yWindow="2715" windowWidth="16770" windowHeight="15345" xr2:uid="{F42F43B3-C9C7-49B5-A63B-84B6B370C241}"/>
   </bookViews>
   <sheets>
     <sheet name="levoglucosan" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t>time</t>
   </si>
@@ -368,13 +368,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA32E4AB-18F3-4BB4-AF4F-4B3B28085FDA}">
-  <dimension ref="A1:L529"/>
+  <dimension ref="A1:M529"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="12" max="12" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -400,10 +400,13 @@
         <v>7</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.02</v>
       </c>
@@ -429,10 +432,13 @@
         <v>40</v>
       </c>
       <c r="L2">
+        <v>1.56</v>
+      </c>
+      <c r="M2">
         <v>0.125</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0.03</v>
       </c>
@@ -440,7 +446,7 @@
         <v>11967</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0.05</v>
       </c>
@@ -448,7 +454,7 @@
         <v>12008.17</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -457,7 +463,7 @@
       </c>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.08</v>
       </c>
@@ -466,7 +472,7 @@
       </c>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0.1</v>
       </c>
@@ -474,7 +480,7 @@
         <v>11947.87</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.12</v>
       </c>
@@ -482,7 +488,7 @@
         <v>11974.44</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0.13</v>
       </c>
@@ -490,7 +496,7 @@
         <v>11997.88</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>0.15</v>
       </c>
@@ -498,7 +504,7 @@
         <v>11973.03</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>0.17</v>
       </c>
@@ -506,7 +512,7 @@
         <v>11963.77</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0.19</v>
       </c>
@@ -514,7 +520,7 @@
         <v>11976.52</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>0.2</v>
       </c>
@@ -522,7 +528,7 @@
         <v>11974.99</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0.22</v>
       </c>
@@ -530,7 +536,7 @@
         <v>11976.19</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0.24</v>
       </c>
@@ -538,7 +544,7 @@
         <v>12054.6</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>0.25</v>
       </c>

</xml_diff>